<commit_message>
Move gitignore to root and remove venv
</commit_message>
<xml_diff>
--- a/backend/API_CheckList.xlsx
+++ b/backend/API_CheckList.xlsx
@@ -1,21 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="25330"/>
-  <workbookPr/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28014"/>
+  <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\PCOS_Risk_Assessment_System\backend\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\megah\Desktop\PCOS Application\backend\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AE8A8465-F719-4B68-B1B5-078C7E8A0EE6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{465EDE6D-EFD4-4574-980A-C8C81CDC0890}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{FB716B8F-6B6F-4BC2-BD7E-9FF071F42922}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{FB716B8F-6B6F-4BC2-BD7E-9FF071F42922}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -23,9 +23,12 @@
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
         <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
         <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
         <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
   </extLst>
@@ -219,7 +222,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -270,7 +273,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
@@ -290,17 +293,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1">
-      <extLst>
-        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
-          <xfpb:xfComplement i="0"/>
-        </ext>
-      </extLst>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -663,38 +655,38 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4F7A5DDD-25D9-475A-8AF5-99E140546EAF}">
   <dimension ref="A1:E59"/>
-  <sheetFormatPr defaultRowHeight="13.8"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="42" customWidth="1"/>
-    <col min="2" max="2" width="15.3984375" customWidth="1"/>
-    <col min="3" max="3" width="37.09765625" customWidth="1"/>
-    <col min="4" max="4" width="11.19921875" customWidth="1"/>
+    <col min="2" max="2" width="15.44140625" customWidth="1"/>
+    <col min="3" max="3" width="37.109375" customWidth="1"/>
+    <col min="4" max="4" width="11.21875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="14.4" customHeight="1">
-      <c r="A1" s="11" t="s">
+    <row r="1" spans="1:5" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="8" t="s">
         <v>19</v>
       </c>
-      <c r="B1" s="11"/>
-      <c r="C1" s="11"/>
-      <c r="D1" s="11"/>
-      <c r="E1" s="11"/>
-    </row>
-    <row r="2" spans="1:5" ht="14.4" customHeight="1">
-      <c r="A2" s="11"/>
-      <c r="B2" s="11"/>
-      <c r="C2" s="11"/>
-      <c r="D2" s="11"/>
-      <c r="E2" s="11"/>
-    </row>
-    <row r="3" spans="1:5" ht="14.4" customHeight="1">
-      <c r="A3" s="11"/>
-      <c r="B3" s="11"/>
-      <c r="C3" s="11"/>
-      <c r="D3" s="11"/>
-      <c r="E3" s="11"/>
-    </row>
-    <row r="4" spans="1:5">
+      <c r="B1" s="8"/>
+      <c r="C1" s="8"/>
+      <c r="D1" s="8"/>
+      <c r="E1" s="8"/>
+    </row>
+    <row r="2" spans="1:5" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="8"/>
+      <c r="B2" s="8"/>
+      <c r="C2" s="8"/>
+      <c r="D2" s="8"/>
+      <c r="E2" s="8"/>
+    </row>
+    <row r="3" spans="1:5" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="8"/>
+      <c r="B3" s="8"/>
+      <c r="C3" s="8"/>
+      <c r="D3" s="8"/>
+      <c r="E3" s="8"/>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
         <v>0</v>
       </c>
@@ -708,7 +700,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:5">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -722,7 +714,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:5">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>10</v>
       </c>
@@ -736,7 +728,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:5">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A7" s="3" t="s">
         <v>11</v>
       </c>
@@ -750,7 +742,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:5">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A8" s="3" t="s">
         <v>12</v>
       </c>
@@ -764,7 +756,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:5">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A9" s="3" t="s">
         <v>13</v>
       </c>
@@ -778,67 +770,63 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:5" ht="27.6">
-      <c r="A10" s="6" t="s">
+    <row r="10" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
         <v>14</v>
       </c>
-      <c r="B10" s="6" t="s">
+      <c r="B10" t="s">
         <v>15</v>
       </c>
-      <c r="C10" s="7" t="s">
+      <c r="C10" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="D10" s="8" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5">
+      <c r="D10" s="2" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>20</v>
       </c>
       <c r="B11" t="s">
         <v>4</v>
       </c>
-      <c r="C11" s="6" t="s">
+      <c r="C11" t="s">
         <v>21</v>
       </c>
       <c r="D11" s="2" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:5">
-      <c r="C12" s="6"/>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
       <c r="D12" s="2" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:5">
-      <c r="C13" s="6"/>
-    </row>
-    <row r="14" spans="1:5">
-      <c r="A14" s="11" t="s">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A14" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="B14" s="11"/>
-      <c r="C14" s="11"/>
-      <c r="D14" s="11"/>
-      <c r="E14" s="11"/>
-    </row>
-    <row r="15" spans="1:5">
-      <c r="A15" s="11"/>
-      <c r="B15" s="11"/>
-      <c r="C15" s="11"/>
-      <c r="D15" s="11"/>
-      <c r="E15" s="11"/>
-    </row>
-    <row r="16" spans="1:5">
-      <c r="A16" s="11"/>
-      <c r="B16" s="11"/>
-      <c r="C16" s="11"/>
-      <c r="D16" s="11"/>
-      <c r="E16" s="11"/>
-    </row>
-    <row r="17" spans="1:5">
+      <c r="B14" s="8"/>
+      <c r="C14" s="8"/>
+      <c r="D14" s="8"/>
+      <c r="E14" s="8"/>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A15" s="8"/>
+      <c r="B15" s="8"/>
+      <c r="C15" s="8"/>
+      <c r="D15" s="8"/>
+      <c r="E15" s="8"/>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A16" s="8"/>
+      <c r="B16" s="8"/>
+      <c r="C16" s="8"/>
+      <c r="D16" s="8"/>
+      <c r="E16" s="8"/>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A17" s="1" t="s">
         <v>0</v>
       </c>
@@ -852,7 +840,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="18" spans="1:5">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>17</v>
       </c>
@@ -866,7 +854,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:5">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>30</v>
       </c>
@@ -880,7 +868,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:5">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>30</v>
       </c>
@@ -894,30 +882,30 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:5">
-      <c r="A23" s="11" t="s">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A23" s="8" t="s">
         <v>28</v>
       </c>
-      <c r="B23" s="11"/>
-      <c r="C23" s="11"/>
-      <c r="D23" s="11"/>
-      <c r="E23" s="11"/>
-    </row>
-    <row r="24" spans="1:5">
-      <c r="A24" s="11"/>
-      <c r="B24" s="11"/>
-      <c r="C24" s="11"/>
-      <c r="D24" s="11"/>
-      <c r="E24" s="11"/>
-    </row>
-    <row r="25" spans="1:5">
-      <c r="A25" s="11"/>
-      <c r="B25" s="11"/>
-      <c r="C25" s="11"/>
-      <c r="D25" s="11"/>
-      <c r="E25" s="11"/>
-    </row>
-    <row r="26" spans="1:5">
+      <c r="B23" s="8"/>
+      <c r="C23" s="8"/>
+      <c r="D23" s="8"/>
+      <c r="E23" s="8"/>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A24" s="8"/>
+      <c r="B24" s="8"/>
+      <c r="C24" s="8"/>
+      <c r="D24" s="8"/>
+      <c r="E24" s="8"/>
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A25" s="8"/>
+      <c r="B25" s="8"/>
+      <c r="C25" s="8"/>
+      <c r="D25" s="8"/>
+      <c r="E25" s="8"/>
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A26" s="1" t="s">
         <v>0</v>
       </c>
@@ -931,7 +919,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="27" spans="1:5">
+    <row r="27" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>36</v>
       </c>
@@ -945,7 +933,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="1:5">
+    <row r="28" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>36</v>
       </c>
@@ -959,21 +947,21 @@
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="1:5" ht="27.6">
+    <row r="29" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>36</v>
       </c>
-      <c r="B29" s="9" t="s">
+      <c r="B29" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="C29" s="9" t="s">
+      <c r="C29" s="6" t="s">
         <v>50</v>
       </c>
       <c r="D29" s="2" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="30" spans="1:5">
+    <row r="30" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>37</v>
       </c>
@@ -987,7 +975,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="1:5">
+    <row r="31" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
         <v>37</v>
       </c>
@@ -1001,7 +989,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="32" spans="1:5">
+    <row r="32" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
         <v>37</v>
       </c>
@@ -1015,30 +1003,30 @@
         <v>0</v>
       </c>
     </row>
-    <row r="35" spans="1:5">
-      <c r="A35" s="11" t="s">
+    <row r="35" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A35" s="8" t="s">
         <v>39</v>
       </c>
-      <c r="B35" s="11"/>
-      <c r="C35" s="11"/>
-      <c r="D35" s="11"/>
-      <c r="E35" s="11"/>
-    </row>
-    <row r="36" spans="1:5">
-      <c r="A36" s="11"/>
-      <c r="B36" s="11"/>
-      <c r="C36" s="11"/>
-      <c r="D36" s="11"/>
-      <c r="E36" s="11"/>
-    </row>
-    <row r="37" spans="1:5">
-      <c r="A37" s="11"/>
-      <c r="B37" s="11"/>
-      <c r="C37" s="11"/>
-      <c r="D37" s="11"/>
-      <c r="E37" s="11"/>
-    </row>
-    <row r="38" spans="1:5">
+      <c r="B35" s="8"/>
+      <c r="C35" s="8"/>
+      <c r="D35" s="8"/>
+      <c r="E35" s="8"/>
+    </row>
+    <row r="36" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A36" s="8"/>
+      <c r="B36" s="8"/>
+      <c r="C36" s="8"/>
+      <c r="D36" s="8"/>
+      <c r="E36" s="8"/>
+    </row>
+    <row r="37" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A37" s="8"/>
+      <c r="B37" s="8"/>
+      <c r="C37" s="8"/>
+      <c r="D37" s="8"/>
+      <c r="E37" s="8"/>
+    </row>
+    <row r="38" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A38" s="1" t="s">
         <v>0</v>
       </c>
@@ -1052,7 +1040,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="39" spans="1:5" ht="27.6">
+    <row r="39" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A39" s="3" t="s">
         <v>40</v>
       </c>
@@ -1066,7 +1054,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="40" spans="1:5">
+    <row r="40" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
         <v>40</v>
       </c>
@@ -1080,7 +1068,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="41" spans="1:5">
+    <row r="41" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
         <v>44</v>
       </c>
@@ -1094,7 +1082,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="42" spans="1:5">
+    <row r="42" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
         <v>44</v>
       </c>
@@ -1108,7 +1096,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="43" spans="1:5">
+    <row r="43" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
         <v>44</v>
       </c>
@@ -1122,7 +1110,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="44" spans="1:5" ht="27.6">
+    <row r="44" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A44" s="3" t="s">
         <v>54</v>
       </c>
@@ -1136,7 +1124,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="45" spans="1:5">
+    <row r="45" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A45" s="3"/>
       <c r="B45" s="5"/>
       <c r="C45" s="5"/>
@@ -1144,30 +1132,30 @@
         <v>0</v>
       </c>
     </row>
-    <row r="47" spans="1:5">
-      <c r="A47" s="11" t="s">
+    <row r="47" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A47" s="8" t="s">
         <v>53</v>
       </c>
-      <c r="B47" s="11"/>
-      <c r="C47" s="11"/>
-      <c r="D47" s="11"/>
-      <c r="E47" s="11"/>
-    </row>
-    <row r="48" spans="1:5">
-      <c r="A48" s="11"/>
-      <c r="B48" s="11"/>
-      <c r="C48" s="11"/>
-      <c r="D48" s="11"/>
-      <c r="E48" s="11"/>
-    </row>
-    <row r="49" spans="1:5">
-      <c r="A49" s="11"/>
-      <c r="B49" s="11"/>
-      <c r="C49" s="11"/>
-      <c r="D49" s="11"/>
-      <c r="E49" s="11"/>
-    </row>
-    <row r="50" spans="1:5">
+      <c r="B47" s="8"/>
+      <c r="C47" s="8"/>
+      <c r="D47" s="8"/>
+      <c r="E47" s="8"/>
+    </row>
+    <row r="48" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A48" s="8"/>
+      <c r="B48" s="8"/>
+      <c r="C48" s="8"/>
+      <c r="D48" s="8"/>
+      <c r="E48" s="8"/>
+    </row>
+    <row r="49" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A49" s="8"/>
+      <c r="B49" s="8"/>
+      <c r="C49" s="8"/>
+      <c r="D49" s="8"/>
+      <c r="E49" s="8"/>
+    </row>
+    <row r="50" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A50" s="1" t="s">
         <v>0</v>
       </c>
@@ -1181,44 +1169,44 @@
         <v>3</v>
       </c>
     </row>
-    <row r="51" spans="1:5" ht="27.6">
+    <row r="51" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
         <v>51</v>
       </c>
       <c r="B51" t="s">
         <v>25</v>
       </c>
-      <c r="C51" s="10" t="s">
+      <c r="C51" s="7" t="s">
         <v>52</v>
       </c>
       <c r="D51" s="2" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="54" spans="1:5">
-      <c r="A54" s="11" t="s">
+    <row r="54" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A54" s="8" t="s">
         <v>57</v>
       </c>
-      <c r="B54" s="11"/>
-      <c r="C54" s="11"/>
-      <c r="D54" s="11"/>
-      <c r="E54" s="11"/>
-    </row>
-    <row r="55" spans="1:5">
-      <c r="A55" s="11"/>
-      <c r="B55" s="11"/>
-      <c r="C55" s="11"/>
-      <c r="D55" s="11"/>
-      <c r="E55" s="11"/>
-    </row>
-    <row r="56" spans="1:5">
-      <c r="A56" s="11"/>
-      <c r="B56" s="11"/>
-      <c r="C56" s="11"/>
-      <c r="D56" s="11"/>
-      <c r="E56" s="11"/>
-    </row>
-    <row r="57" spans="1:5">
+      <c r="B54" s="8"/>
+      <c r="C54" s="8"/>
+      <c r="D54" s="8"/>
+      <c r="E54" s="8"/>
+    </row>
+    <row r="55" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A55" s="8"/>
+      <c r="B55" s="8"/>
+      <c r="C55" s="8"/>
+      <c r="D55" s="8"/>
+      <c r="E55" s="8"/>
+    </row>
+    <row r="56" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A56" s="8"/>
+      <c r="B56" s="8"/>
+      <c r="C56" s="8"/>
+      <c r="D56" s="8"/>
+      <c r="E56" s="8"/>
+    </row>
+    <row r="57" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A57" s="1" t="s">
         <v>0</v>
       </c>
@@ -1232,21 +1220,21 @@
         <v>3</v>
       </c>
     </row>
-    <row r="58" spans="1:5" ht="27.6">
+    <row r="58" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A58" t="s">
         <v>49</v>
       </c>
       <c r="B58" t="s">
         <v>25</v>
       </c>
-      <c r="C58" s="10" t="s">
+      <c r="C58" s="7" t="s">
         <v>52</v>
       </c>
       <c r="D58" s="2" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="59" spans="1:5">
+    <row r="59" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A59" s="3" t="s">
         <v>58</v>
       </c>

</xml_diff>

<commit_message>
forgot password apis created
</commit_message>
<xml_diff>
--- a/backend/API_CheckList.xlsx
+++ b/backend/API_CheckList.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\megah\Desktop\PCOS Application\backend\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{465EDE6D-EFD4-4574-980A-C8C81CDC0890}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E7FD810E-4C76-4ADA-A4A1-F7C0E427815D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{FB716B8F-6B6F-4BC2-BD7E-9FF071F42922}"/>
   </bookViews>
@@ -739,7 +739,7 @@
         <v>5</v>
       </c>
       <c r="D7" s="4" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.3">
@@ -753,7 +753,7 @@
         <v>8</v>
       </c>
       <c r="D8" s="4" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.3">
@@ -767,7 +767,7 @@
         <v>22</v>
       </c>
       <c r="D9" s="4" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="10" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
refresh token endpoint with token rotation implemented
</commit_message>
<xml_diff>
--- a/backend/API_CheckList.xlsx
+++ b/backend/API_CheckList.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="25330"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28014"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\PCOS_Risk_Assessment_System\backend\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\megah\Desktop\PCOS Application\backend\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{73F00982-E77E-450A-95A5-6045219EDED6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9F8662D8-08A2-4F2B-A098-57A0F2A3AC8B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{FB716B8F-6B6F-4BC2-BD7E-9FF071F42922}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{FB716B8F-6B6F-4BC2-BD7E-9FF071F42922}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -216,7 +216,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -649,15 +649,15 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4F7A5DDD-25D9-475A-8AF5-99E140546EAF}">
   <dimension ref="A1:E59"/>
-  <sheetFormatPr defaultRowHeight="13.8"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="42" customWidth="1"/>
-    <col min="2" max="2" width="15.3984375" customWidth="1"/>
-    <col min="3" max="3" width="37.09765625" customWidth="1"/>
-    <col min="4" max="4" width="11.19921875" customWidth="1"/>
+    <col min="2" max="2" width="15.44140625" customWidth="1"/>
+    <col min="3" max="3" width="37.109375" customWidth="1"/>
+    <col min="4" max="4" width="11.21875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="14.4" customHeight="1">
+    <row r="1" spans="1:5" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="8" t="s">
         <v>19</v>
       </c>
@@ -666,21 +666,21 @@
       <c r="D1" s="8"/>
       <c r="E1" s="8"/>
     </row>
-    <row r="2" spans="1:5" ht="14.4" customHeight="1">
+    <row r="2" spans="1:5" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="8"/>
       <c r="B2" s="8"/>
       <c r="C2" s="8"/>
       <c r="D2" s="8"/>
       <c r="E2" s="8"/>
     </row>
-    <row r="3" spans="1:5" ht="14.4" customHeight="1">
+    <row r="3" spans="1:5" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="8"/>
       <c r="B3" s="8"/>
       <c r="C3" s="8"/>
       <c r="D3" s="8"/>
       <c r="E3" s="8"/>
     </row>
-    <row r="4" spans="1:5">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
         <v>0</v>
       </c>
@@ -694,7 +694,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:5">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -708,7 +708,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:5">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>10</v>
       </c>
@@ -722,7 +722,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:5">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A7" s="3" t="s">
         <v>11</v>
       </c>
@@ -736,7 +736,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:5">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A8" s="3" t="s">
         <v>12</v>
       </c>
@@ -750,7 +750,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:5">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A9" s="3" t="s">
         <v>13</v>
       </c>
@@ -764,7 +764,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:5" ht="27.6">
+    <row r="10" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>14</v>
       </c>
@@ -775,10 +775,10 @@
         <v>16</v>
       </c>
       <c r="D10" s="2" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>20</v>
       </c>
@@ -789,15 +789,10 @@
         <v>21</v>
       </c>
       <c r="D11" s="2" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5">
-      <c r="D12" s="2" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="14" spans="1:5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A14" s="8" t="s">
         <v>18</v>
       </c>
@@ -806,21 +801,21 @@
       <c r="D14" s="8"/>
       <c r="E14" s="8"/>
     </row>
-    <row r="15" spans="1:5">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A15" s="8"/>
       <c r="B15" s="8"/>
       <c r="C15" s="8"/>
       <c r="D15" s="8"/>
       <c r="E15" s="8"/>
     </row>
-    <row r="16" spans="1:5">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A16" s="8"/>
       <c r="B16" s="8"/>
       <c r="C16" s="8"/>
       <c r="D16" s="8"/>
       <c r="E16" s="8"/>
     </row>
-    <row r="17" spans="1:5">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A17" s="1" t="s">
         <v>0</v>
       </c>
@@ -834,7 +829,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="18" spans="1:5">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>17</v>
       </c>
@@ -848,7 +843,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="1:5">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>30</v>
       </c>
@@ -862,7 +857,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="20" spans="1:5">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>30</v>
       </c>
@@ -876,7 +871,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="23" spans="1:5">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A23" s="8" t="s">
         <v>28</v>
       </c>
@@ -885,21 +880,21 @@
       <c r="D23" s="8"/>
       <c r="E23" s="8"/>
     </row>
-    <row r="24" spans="1:5">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A24" s="8"/>
       <c r="B24" s="8"/>
       <c r="C24" s="8"/>
       <c r="D24" s="8"/>
       <c r="E24" s="8"/>
     </row>
-    <row r="25" spans="1:5">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A25" s="8"/>
       <c r="B25" s="8"/>
       <c r="C25" s="8"/>
       <c r="D25" s="8"/>
       <c r="E25" s="8"/>
     </row>
-    <row r="26" spans="1:5">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A26" s="1" t="s">
         <v>0</v>
       </c>
@@ -913,7 +908,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="27" spans="1:5">
+    <row r="27" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>36</v>
       </c>
@@ -927,7 +922,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="28" spans="1:5">
+    <row r="28" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>36</v>
       </c>
@@ -941,7 +936,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="29" spans="1:5" ht="27.6">
+    <row r="29" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>36</v>
       </c>
@@ -955,7 +950,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="30" spans="1:5">
+    <row r="30" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>37</v>
       </c>
@@ -969,7 +964,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="31" spans="1:5">
+    <row r="31" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
         <v>37</v>
       </c>
@@ -983,7 +978,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="32" spans="1:5">
+    <row r="32" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
         <v>37</v>
       </c>
@@ -997,7 +992,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="35" spans="1:5">
+    <row r="35" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A35" s="8" t="s">
         <v>39</v>
       </c>
@@ -1006,21 +1001,21 @@
       <c r="D35" s="8"/>
       <c r="E35" s="8"/>
     </row>
-    <row r="36" spans="1:5">
+    <row r="36" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A36" s="8"/>
       <c r="B36" s="8"/>
       <c r="C36" s="8"/>
       <c r="D36" s="8"/>
       <c r="E36" s="8"/>
     </row>
-    <row r="37" spans="1:5">
+    <row r="37" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A37" s="8"/>
       <c r="B37" s="8"/>
       <c r="C37" s="8"/>
       <c r="D37" s="8"/>
       <c r="E37" s="8"/>
     </row>
-    <row r="38" spans="1:5">
+    <row r="38" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A38" s="1" t="s">
         <v>0</v>
       </c>
@@ -1034,7 +1029,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="39" spans="1:5" ht="27.6">
+    <row r="39" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A39" s="3" t="s">
         <v>40</v>
       </c>
@@ -1048,7 +1043,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="40" spans="1:5">
+    <row r="40" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
         <v>40</v>
       </c>
@@ -1062,7 +1057,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="41" spans="1:5">
+    <row r="41" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
         <v>44</v>
       </c>
@@ -1076,10 +1071,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="42" spans="1:5">
-      <c r="D42" s="2"/>
-    </row>
-    <row r="43" spans="1:5">
+    <row r="43" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
         <v>44</v>
       </c>
@@ -1093,7 +1085,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="44" spans="1:5" ht="27.6">
+    <row r="44" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A44" s="3" t="s">
         <v>53</v>
       </c>
@@ -1107,7 +1099,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="45" spans="1:5">
+    <row r="45" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A45" s="3"/>
       <c r="B45" s="5"/>
       <c r="C45" s="5"/>
@@ -1115,7 +1107,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="47" spans="1:5">
+    <row r="47" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A47" s="8" t="s">
         <v>52</v>
       </c>
@@ -1124,21 +1116,21 @@
       <c r="D47" s="8"/>
       <c r="E47" s="8"/>
     </row>
-    <row r="48" spans="1:5">
+    <row r="48" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A48" s="8"/>
       <c r="B48" s="8"/>
       <c r="C48" s="8"/>
       <c r="D48" s="8"/>
       <c r="E48" s="8"/>
     </row>
-    <row r="49" spans="1:5">
+    <row r="49" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A49" s="8"/>
       <c r="B49" s="8"/>
       <c r="C49" s="8"/>
       <c r="D49" s="8"/>
       <c r="E49" s="8"/>
     </row>
-    <row r="50" spans="1:5" ht="14.4">
+    <row r="50" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A50" s="1" t="s">
         <v>0</v>
       </c>
@@ -1152,7 +1144,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="51" spans="1:5" ht="27.6">
+    <row r="51" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
         <v>50</v>
       </c>
@@ -1166,7 +1158,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="54" spans="1:5">
+    <row r="54" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A54" s="8" t="s">
         <v>56</v>
       </c>
@@ -1175,21 +1167,21 @@
       <c r="D54" s="8"/>
       <c r="E54" s="8"/>
     </row>
-    <row r="55" spans="1:5">
+    <row r="55" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A55" s="8"/>
       <c r="B55" s="8"/>
       <c r="C55" s="8"/>
       <c r="D55" s="8"/>
       <c r="E55" s="8"/>
     </row>
-    <row r="56" spans="1:5">
+    <row r="56" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A56" s="8"/>
       <c r="B56" s="8"/>
       <c r="C56" s="8"/>
       <c r="D56" s="8"/>
       <c r="E56" s="8"/>
     </row>
-    <row r="57" spans="1:5" ht="14.4">
+    <row r="57" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A57" s="1" t="s">
         <v>0</v>
       </c>
@@ -1203,7 +1195,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="58" spans="1:5" ht="27.6">
+    <row r="58" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A58" t="s">
         <v>48</v>
       </c>
@@ -1217,7 +1209,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="59" spans="1:5">
+    <row r="59" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A59" s="3" t="s">
         <v>57</v>
       </c>

</xml_diff>